<commit_message>
Mise à jour automatique des fichiers Eclipse Replication
</commit_message>
<xml_diff>
--- a/static/assets/LastUpdatedWithPredictions.xlsx
+++ b/static/assets/LastUpdatedWithPredictions.xlsx
@@ -18889,28 +18889,28 @@
         <v>537</v>
       </c>
       <c r="B529">
-        <v>1.026573151777872</v>
+        <v>1.025325869854519</v>
       </c>
       <c r="C529">
-        <v>0.6185959320803529</v>
+        <v>0.6186157200557788</v>
       </c>
       <c r="D529">
-        <v>28.72867808787964</v>
+        <v>28.69519774291497</v>
       </c>
       <c r="E529">
-        <v>68701.77</v>
+        <v>68629.9599760374</v>
       </c>
       <c r="F529">
-        <v>0.5333</v>
+        <v>0.5243</v>
       </c>
       <c r="G529">
-        <v>22.02135163</v>
+        <v>21.76869686</v>
       </c>
       <c r="H529">
         <v>0.89570088967656</v>
       </c>
       <c r="I529">
-        <v>-1.361275679537277</v>
+        <v>-0.1365282441126214</v>
       </c>
       <c r="J529">
         <v>0.3104479610919952</v>

</xml_diff>